<commit_message>
feat: 7-tab Excel import template — phases, departments, RU labels, mandatory fields
</commit_message>
<xml_diff>
--- a/test-data/test-import-3tab.xlsx
+++ b/test-data/test-import-3tab.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Заказы" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Маршруты" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заказы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Маршруты" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -607,7 +607,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>assembly</t>
@@ -784,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -805,30 +804,40 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Станок</t>
+          <t>Ресурс</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Этап</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Подразделение</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Длит.,ч</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Предш. оп.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Доп. материал</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Расход</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Вых. годного</t>
         </is>
@@ -837,17 +846,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Сборка редуктора</t>
+          <t>Сборка корпуса</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -856,14 +863,23 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Цех №5</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
+      <c r="K2" t="n">
+        <v>0.98</v>
       </c>
     </row>
     <row r="3">
@@ -874,69 +890,75 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Контроль</t>
+          <t>Сборка редуктора</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Контролёр</t>
+          <t>Слесарь</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Цех №2</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Сборка корпуса</t>
+          <t>Контроль</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Слесарь</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Контролёр</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
       <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="n">
-        <v>0.98</v>
+      <c r="K4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -946,27 +968,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Токарная</t>
+          <t>Сборка корпуса</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Токарь</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Сталь 40Х</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.95</v>
+          <t>Слесарь</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.98</v>
       </c>
     </row>
     <row r="6">
@@ -977,30 +994,65 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Токарная</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Токарь</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Сталь 40Х</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1.1.2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Шлифовка</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Шлифовщик</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="G7" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H7" t="n">
         <v>1</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K7" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>